<commit_message>
Add English Assessment Score Sheet layout
</commit_message>
<xml_diff>
--- a/English_Assessment_Score_Sheet.xlsx
+++ b/English_Assessment_Score_Sheet.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,7 +35,7 @@
     </font>
     <font>
       <b val="1"/>
-      <sz val="12"/>
+      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
@@ -45,10 +45,6 @@
     <font>
       <b val="1"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
@@ -86,7 +82,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -99,27 +95,6 @@
       <right style="thin"/>
       <top style="thin"/>
       <bottom style="thin"/>
-    </border>
-    <border>
-      <left style="thin"/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top/>
-      <bottom style="thin"/>
-      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -140,10 +115,10 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -157,7 +132,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -573,7 +548,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Score Entry Sheet - Input scores for each exercise</t>
+          <t>Input scores for each exercise below</t>
         </is>
       </c>
     </row>
@@ -1215,12 +1190,12 @@
     </row>
   </sheetData>
   <mergeCells count="10">
-    <mergeCell ref="A2:AB2"/>
+    <mergeCell ref="A1:AG1"/>
     <mergeCell ref="B4:B5"/>
     <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A2:AG2"/>
     <mergeCell ref="O4:T4"/>
     <mergeCell ref="AG4:AG5"/>
-    <mergeCell ref="A1:AB1"/>
     <mergeCell ref="C4:H4"/>
     <mergeCell ref="U4:Z4"/>
     <mergeCell ref="AA4:AF4"/>

</xml_diff>

<commit_message>
Update English Assessment: 1 essay exercise, named Lexis exercises with max scores, student scores entered
</commit_message>
<xml_diff>
--- a/English_Assessment_Score_Sheet.xlsx
+++ b/English_Assessment_Score_Sheet.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,6 +41,10 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="9"/>
     </font>
     <font>
       <b val="1"/>
@@ -122,7 +126,7 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -132,7 +136,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -500,42 +504,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG12"/>
+  <dimension ref="A1:AC12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="8" customWidth="1" min="12" max="12"/>
-    <col width="8" customWidth="1" min="13" max="13"/>
-    <col width="8" customWidth="1" min="14" max="14"/>
-    <col width="8" customWidth="1" min="15" max="15"/>
-    <col width="8" customWidth="1" min="16" max="16"/>
-    <col width="8" customWidth="1" min="17" max="17"/>
-    <col width="8" customWidth="1" min="18" max="18"/>
-    <col width="8" customWidth="1" min="19" max="19"/>
-    <col width="8" customWidth="1" min="20" max="20"/>
-    <col width="8" customWidth="1" min="21" max="21"/>
-    <col width="8" customWidth="1" min="22" max="22"/>
-    <col width="8" customWidth="1" min="23" max="23"/>
-    <col width="8" customWidth="1" min="24" max="24"/>
-    <col width="8" customWidth="1" min="25" max="25"/>
-    <col width="8" customWidth="1" min="26" max="26"/>
-    <col width="8" customWidth="1" min="27" max="27"/>
-    <col width="8" customWidth="1" min="28" max="28"/>
-    <col width="8" customWidth="1" min="29" max="29"/>
-    <col width="8" customWidth="1" min="30" max="30"/>
-    <col width="8" customWidth="1" min="31" max="31"/>
-    <col width="8" customWidth="1" min="32" max="32"/>
-    <col width="8" customWidth="1" min="33" max="33"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
+    <col width="12" customWidth="1" min="24" max="24"/>
+    <col width="12" customWidth="1" min="25" max="25"/>
+    <col width="12" customWidth="1" min="26" max="26"/>
+    <col width="12" customWidth="1" min="27" max="27"/>
+    <col width="12" customWidth="1" min="28" max="28"/>
+    <col width="12" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -569,51 +569,47 @@
         </is>
       </c>
       <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Comprehension</t>
+        </is>
+      </c>
       <c r="F4" s="5" t="n"/>
       <c r="G4" s="5" t="n"/>
       <c r="H4" s="5" t="n"/>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>Comprehension</t>
-        </is>
-      </c>
+      <c r="I4" s="5" t="n"/>
       <c r="J4" s="5" t="n"/>
-      <c r="K4" s="5" t="n"/>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
       <c r="L4" s="5" t="n"/>
       <c r="M4" s="5" t="n"/>
       <c r="N4" s="5" t="n"/>
-      <c r="O4" s="4" t="inlineStr">
-        <is>
-          <t>Summary</t>
-        </is>
-      </c>
+      <c r="O4" s="5" t="n"/>
       <c r="P4" s="5" t="n"/>
-      <c r="Q4" s="5" t="n"/>
+      <c r="Q4" s="4" t="inlineStr">
+        <is>
+          <t>Lexis and Structure</t>
+        </is>
+      </c>
       <c r="R4" s="5" t="n"/>
       <c r="S4" s="5" t="n"/>
       <c r="T4" s="5" t="n"/>
-      <c r="U4" s="4" t="inlineStr">
-        <is>
-          <t>Lexis and Structure</t>
-        </is>
-      </c>
+      <c r="U4" s="5" t="n"/>
       <c r="V4" s="5" t="n"/>
-      <c r="W4" s="5" t="n"/>
+      <c r="W4" s="4" t="inlineStr">
+        <is>
+          <t>Oral English</t>
+        </is>
+      </c>
       <c r="X4" s="5" t="n"/>
       <c r="Y4" s="5" t="n"/>
       <c r="Z4" s="5" t="n"/>
-      <c r="AA4" s="4" t="inlineStr">
-        <is>
-          <t>Oral English</t>
-        </is>
-      </c>
+      <c r="AA4" s="5" t="n"/>
       <c r="AB4" s="5" t="n"/>
-      <c r="AC4" s="5" t="n"/>
-      <c r="AD4" s="5" t="n"/>
-      <c r="AE4" s="5" t="n"/>
-      <c r="AF4" s="5" t="n"/>
-      <c r="AG4" s="6" t="inlineStr">
+      <c r="AC4" s="6" t="inlineStr">
         <is>
           <t>GRAND
 TOTAL</t>
@@ -625,155 +621,141 @@
       <c r="B5" s="7" t="n"/>
       <c r="C5" s="8" t="inlineStr">
         <is>
+          <t>Essay
+(50)</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
           <t>Ex 1</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="F5" s="8" t="inlineStr">
         <is>
           <t>Ex 2</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="G5" s="8" t="inlineStr">
         <is>
           <t>Ex 3</t>
         </is>
       </c>
-      <c r="F5" s="8" t="inlineStr">
+      <c r="H5" s="8" t="inlineStr">
         <is>
           <t>Ex 4</t>
         </is>
       </c>
-      <c r="G5" s="8" t="inlineStr">
+      <c r="I5" s="8" t="inlineStr">
         <is>
           <t>Ex 5</t>
         </is>
       </c>
-      <c r="H5" s="9" t="inlineStr">
+      <c r="J5" s="9" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="I5" s="8" t="inlineStr">
+      <c r="K5" s="8" t="inlineStr">
         <is>
           <t>Ex 1</t>
         </is>
       </c>
-      <c r="J5" s="8" t="inlineStr">
+      <c r="L5" s="8" t="inlineStr">
         <is>
           <t>Ex 2</t>
         </is>
       </c>
-      <c r="K5" s="8" t="inlineStr">
+      <c r="M5" s="8" t="inlineStr">
         <is>
           <t>Ex 3</t>
         </is>
       </c>
-      <c r="L5" s="8" t="inlineStr">
+      <c r="N5" s="8" t="inlineStr">
         <is>
           <t>Ex 4</t>
         </is>
       </c>
-      <c r="M5" s="8" t="inlineStr">
+      <c r="O5" s="8" t="inlineStr">
         <is>
           <t>Ex 5</t>
         </is>
       </c>
-      <c r="N5" s="9" t="inlineStr">
+      <c r="P5" s="9" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="O5" s="8" t="inlineStr">
+      <c r="Q5" s="8" t="inlineStr">
+        <is>
+          <t>Adjectives
+(43)</t>
+        </is>
+      </c>
+      <c r="R5" s="8" t="inlineStr">
+        <is>
+          <t>Word Registers
+(50)</t>
+        </is>
+      </c>
+      <c r="S5" s="8" t="inlineStr">
+        <is>
+          <t>Prepositions
+(42)</t>
+        </is>
+      </c>
+      <c r="T5" s="8" t="inlineStr">
+        <is>
+          <t>Pronouns
+(18)</t>
+        </is>
+      </c>
+      <c r="U5" s="8" t="inlineStr">
+        <is>
+          <t>Question Tags
+(30)</t>
+        </is>
+      </c>
+      <c r="V5" s="9" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="W5" s="8" t="inlineStr">
         <is>
           <t>Ex 1</t>
         </is>
       </c>
-      <c r="P5" s="8" t="inlineStr">
+      <c r="X5" s="8" t="inlineStr">
         <is>
           <t>Ex 2</t>
         </is>
       </c>
-      <c r="Q5" s="8" t="inlineStr">
+      <c r="Y5" s="8" t="inlineStr">
         <is>
           <t>Ex 3</t>
         </is>
       </c>
-      <c r="R5" s="8" t="inlineStr">
+      <c r="Z5" s="8" t="inlineStr">
         <is>
           <t>Ex 4</t>
         </is>
       </c>
-      <c r="S5" s="8" t="inlineStr">
+      <c r="AA5" s="8" t="inlineStr">
         <is>
           <t>Ex 5</t>
         </is>
       </c>
-      <c r="T5" s="9" t="inlineStr">
+      <c r="AB5" s="9" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="U5" s="8" t="inlineStr">
-        <is>
-          <t>Ex 1</t>
-        </is>
-      </c>
-      <c r="V5" s="8" t="inlineStr">
-        <is>
-          <t>Ex 2</t>
-        </is>
-      </c>
-      <c r="W5" s="8" t="inlineStr">
-        <is>
-          <t>Ex 3</t>
-        </is>
-      </c>
-      <c r="X5" s="8" t="inlineStr">
-        <is>
-          <t>Ex 4</t>
-        </is>
-      </c>
-      <c r="Y5" s="8" t="inlineStr">
-        <is>
-          <t>Ex 5</t>
-        </is>
-      </c>
-      <c r="Z5" s="9" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="AA5" s="8" t="inlineStr">
-        <is>
-          <t>Ex 1</t>
-        </is>
-      </c>
-      <c r="AB5" s="8" t="inlineStr">
-        <is>
-          <t>Ex 2</t>
-        </is>
-      </c>
-      <c r="AC5" s="8" t="inlineStr">
-        <is>
-          <t>Ex 3</t>
-        </is>
-      </c>
-      <c r="AD5" s="8" t="inlineStr">
-        <is>
-          <t>Ex 4</t>
-        </is>
-      </c>
-      <c r="AE5" s="8" t="inlineStr">
-        <is>
-          <t>Ex 5</t>
-        </is>
-      </c>
-      <c r="AF5" s="9" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="AG5" s="10" t="n"/>
+      <c r="AC5" s="10" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="11" t="n">
@@ -785,52 +767,48 @@
         </is>
       </c>
       <c r="C6" s="11" t="n"/>
-      <c r="D6" s="11" t="n"/>
+      <c r="D6" s="13">
+        <f>SUM(C6:C6)</f>
+        <v/>
+      </c>
       <c r="E6" s="11" t="n"/>
       <c r="F6" s="11" t="n"/>
       <c r="G6" s="11" t="n"/>
-      <c r="H6" s="13">
-        <f>SUM(C6:G6)</f>
-        <v/>
-      </c>
+      <c r="H6" s="11" t="n"/>
       <c r="I6" s="11" t="n"/>
-      <c r="J6" s="11" t="n"/>
+      <c r="J6" s="13">
+        <f>SUM(E6:I6)</f>
+        <v/>
+      </c>
       <c r="K6" s="11" t="n"/>
       <c r="L6" s="11" t="n"/>
       <c r="M6" s="11" t="n"/>
-      <c r="N6" s="13">
-        <f>SUM(I6:M6)</f>
-        <v/>
-      </c>
+      <c r="N6" s="11" t="n"/>
       <c r="O6" s="11" t="n"/>
-      <c r="P6" s="11" t="n"/>
+      <c r="P6" s="13">
+        <f>SUM(K6:O6)</f>
+        <v/>
+      </c>
       <c r="Q6" s="11" t="n"/>
       <c r="R6" s="11" t="n"/>
       <c r="S6" s="11" t="n"/>
-      <c r="T6" s="13">
-        <f>SUM(O6:S6)</f>
-        <v/>
-      </c>
+      <c r="T6" s="11" t="n"/>
       <c r="U6" s="11" t="n"/>
-      <c r="V6" s="11" t="n"/>
+      <c r="V6" s="13">
+        <f>SUM(Q6:U6)</f>
+        <v/>
+      </c>
       <c r="W6" s="11" t="n"/>
       <c r="X6" s="11" t="n"/>
       <c r="Y6" s="11" t="n"/>
-      <c r="Z6" s="13">
-        <f>SUM(U6:Y6)</f>
-        <v/>
-      </c>
+      <c r="Z6" s="11" t="n"/>
       <c r="AA6" s="11" t="n"/>
-      <c r="AB6" s="11" t="n"/>
-      <c r="AC6" s="11" t="n"/>
-      <c r="AD6" s="11" t="n"/>
-      <c r="AE6" s="11" t="n"/>
-      <c r="AF6" s="13">
-        <f>SUM(AA6:AE6)</f>
-        <v/>
-      </c>
-      <c r="AG6" s="6">
-        <f>H6+N6+T6+Z6+AF6</f>
+      <c r="AB6" s="13">
+        <f>SUM(W6:AA6)</f>
+        <v/>
+      </c>
+      <c r="AC6" s="6">
+        <f>D6+J6+P6+V6+AB6</f>
         <v/>
       </c>
     </row>
@@ -844,52 +822,48 @@
         </is>
       </c>
       <c r="C7" s="11" t="n"/>
-      <c r="D7" s="11" t="n"/>
+      <c r="D7" s="13">
+        <f>SUM(C7:C7)</f>
+        <v/>
+      </c>
       <c r="E7" s="11" t="n"/>
       <c r="F7" s="11" t="n"/>
       <c r="G7" s="11" t="n"/>
-      <c r="H7" s="13">
-        <f>SUM(C7:G7)</f>
-        <v/>
-      </c>
+      <c r="H7" s="11" t="n"/>
       <c r="I7" s="11" t="n"/>
-      <c r="J7" s="11" t="n"/>
+      <c r="J7" s="13">
+        <f>SUM(E7:I7)</f>
+        <v/>
+      </c>
       <c r="K7" s="11" t="n"/>
       <c r="L7" s="11" t="n"/>
       <c r="M7" s="11" t="n"/>
-      <c r="N7" s="13">
-        <f>SUM(I7:M7)</f>
-        <v/>
-      </c>
+      <c r="N7" s="11" t="n"/>
       <c r="O7" s="11" t="n"/>
-      <c r="P7" s="11" t="n"/>
+      <c r="P7" s="13">
+        <f>SUM(K7:O7)</f>
+        <v/>
+      </c>
       <c r="Q7" s="11" t="n"/>
       <c r="R7" s="11" t="n"/>
       <c r="S7" s="11" t="n"/>
-      <c r="T7" s="13">
-        <f>SUM(O7:S7)</f>
-        <v/>
-      </c>
+      <c r="T7" s="11" t="n"/>
       <c r="U7" s="11" t="n"/>
-      <c r="V7" s="11" t="n"/>
+      <c r="V7" s="13">
+        <f>SUM(Q7:U7)</f>
+        <v/>
+      </c>
       <c r="W7" s="11" t="n"/>
       <c r="X7" s="11" t="n"/>
       <c r="Y7" s="11" t="n"/>
-      <c r="Z7" s="13">
-        <f>SUM(U7:Y7)</f>
-        <v/>
-      </c>
+      <c r="Z7" s="11" t="n"/>
       <c r="AA7" s="11" t="n"/>
-      <c r="AB7" s="11" t="n"/>
-      <c r="AC7" s="11" t="n"/>
-      <c r="AD7" s="11" t="n"/>
-      <c r="AE7" s="11" t="n"/>
-      <c r="AF7" s="13">
-        <f>SUM(AA7:AE7)</f>
-        <v/>
-      </c>
-      <c r="AG7" s="6">
-        <f>H7+N7+T7+Z7+AF7</f>
+      <c r="AB7" s="13">
+        <f>SUM(W7:AA7)</f>
+        <v/>
+      </c>
+      <c r="AC7" s="6">
+        <f>D7+J7+P7+V7+AB7</f>
         <v/>
       </c>
     </row>
@@ -902,53 +876,65 @@
           <t>Olusanya Darasimi</t>
         </is>
       </c>
-      <c r="C8" s="11" t="n"/>
-      <c r="D8" s="11" t="n"/>
-      <c r="E8" s="11" t="n"/>
+      <c r="C8" s="11" t="n">
+        <v>19</v>
+      </c>
+      <c r="D8" s="13">
+        <f>SUM(C8:C8)</f>
+        <v/>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>13</v>
+      </c>
       <c r="F8" s="11" t="n"/>
       <c r="G8" s="11" t="n"/>
-      <c r="H8" s="13">
-        <f>SUM(C8:G8)</f>
-        <v/>
-      </c>
+      <c r="H8" s="11" t="n"/>
       <c r="I8" s="11" t="n"/>
-      <c r="J8" s="11" t="n"/>
-      <c r="K8" s="11" t="n"/>
+      <c r="J8" s="13">
+        <f>SUM(E8:I8)</f>
+        <v/>
+      </c>
+      <c r="K8" s="11" t="n">
+        <v>23</v>
+      </c>
       <c r="L8" s="11" t="n"/>
       <c r="M8" s="11" t="n"/>
-      <c r="N8" s="13">
-        <f>SUM(I8:M8)</f>
-        <v/>
-      </c>
+      <c r="N8" s="11" t="n"/>
       <c r="O8" s="11" t="n"/>
-      <c r="P8" s="11" t="n"/>
-      <c r="Q8" s="11" t="n"/>
-      <c r="R8" s="11" t="n"/>
-      <c r="S8" s="11" t="n"/>
-      <c r="T8" s="13">
-        <f>SUM(O8:S8)</f>
-        <v/>
-      </c>
-      <c r="U8" s="11" t="n"/>
-      <c r="V8" s="11" t="n"/>
+      <c r="P8" s="13">
+        <f>SUM(K8:O8)</f>
+        <v/>
+      </c>
+      <c r="Q8" s="11" t="n">
+        <v>37</v>
+      </c>
+      <c r="R8" s="11" t="n">
+        <v>31</v>
+      </c>
+      <c r="S8" s="11" t="n">
+        <v>31</v>
+      </c>
+      <c r="T8" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="U8" s="11" t="n">
+        <v>24</v>
+      </c>
+      <c r="V8" s="13">
+        <f>SUM(Q8:U8)</f>
+        <v/>
+      </c>
       <c r="W8" s="11" t="n"/>
       <c r="X8" s="11" t="n"/>
       <c r="Y8" s="11" t="n"/>
-      <c r="Z8" s="13">
-        <f>SUM(U8:Y8)</f>
-        <v/>
-      </c>
+      <c r="Z8" s="11" t="n"/>
       <c r="AA8" s="11" t="n"/>
-      <c r="AB8" s="11" t="n"/>
-      <c r="AC8" s="11" t="n"/>
-      <c r="AD8" s="11" t="n"/>
-      <c r="AE8" s="11" t="n"/>
-      <c r="AF8" s="13">
-        <f>SUM(AA8:AE8)</f>
-        <v/>
-      </c>
-      <c r="AG8" s="6">
-        <f>H8+N8+T8+Z8+AF8</f>
+      <c r="AB8" s="13">
+        <f>SUM(W8:AA8)</f>
+        <v/>
+      </c>
+      <c r="AC8" s="6">
+        <f>D8+J8+P8+V8+AB8</f>
         <v/>
       </c>
     </row>
@@ -961,53 +947,63 @@
           <t>Aruna Fuhad</t>
         </is>
       </c>
-      <c r="C9" s="11" t="n"/>
-      <c r="D9" s="11" t="n"/>
+      <c r="C9" s="11" t="n">
+        <v>14</v>
+      </c>
+      <c r="D9" s="13">
+        <f>SUM(C9:C9)</f>
+        <v/>
+      </c>
       <c r="E9" s="11" t="n"/>
       <c r="F9" s="11" t="n"/>
       <c r="G9" s="11" t="n"/>
-      <c r="H9" s="13">
-        <f>SUM(C9:G9)</f>
-        <v/>
-      </c>
+      <c r="H9" s="11" t="n"/>
       <c r="I9" s="11" t="n"/>
-      <c r="J9" s="11" t="n"/>
-      <c r="K9" s="11" t="n"/>
+      <c r="J9" s="13">
+        <f>SUM(E9:I9)</f>
+        <v/>
+      </c>
+      <c r="K9" s="11" t="n">
+        <v>26</v>
+      </c>
       <c r="L9" s="11" t="n"/>
       <c r="M9" s="11" t="n"/>
-      <c r="N9" s="13">
-        <f>SUM(I9:M9)</f>
-        <v/>
-      </c>
+      <c r="N9" s="11" t="n"/>
       <c r="O9" s="11" t="n"/>
-      <c r="P9" s="11" t="n"/>
-      <c r="Q9" s="11" t="n"/>
-      <c r="R9" s="11" t="n"/>
-      <c r="S9" s="11" t="n"/>
-      <c r="T9" s="13">
-        <f>SUM(O9:S9)</f>
-        <v/>
-      </c>
-      <c r="U9" s="11" t="n"/>
-      <c r="V9" s="11" t="n"/>
+      <c r="P9" s="13">
+        <f>SUM(K9:O9)</f>
+        <v/>
+      </c>
+      <c r="Q9" s="11" t="n">
+        <v>34</v>
+      </c>
+      <c r="R9" s="11" t="n">
+        <v>34</v>
+      </c>
+      <c r="S9" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="T9" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="U9" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="V9" s="13">
+        <f>SUM(Q9:U9)</f>
+        <v/>
+      </c>
       <c r="W9" s="11" t="n"/>
       <c r="X9" s="11" t="n"/>
       <c r="Y9" s="11" t="n"/>
-      <c r="Z9" s="13">
-        <f>SUM(U9:Y9)</f>
-        <v/>
-      </c>
+      <c r="Z9" s="11" t="n"/>
       <c r="AA9" s="11" t="n"/>
-      <c r="AB9" s="11" t="n"/>
-      <c r="AC9" s="11" t="n"/>
-      <c r="AD9" s="11" t="n"/>
-      <c r="AE9" s="11" t="n"/>
-      <c r="AF9" s="13">
-        <f>SUM(AA9:AE9)</f>
-        <v/>
-      </c>
-      <c r="AG9" s="6">
-        <f>H9+N9+T9+Z9+AF9</f>
+      <c r="AB9" s="13">
+        <f>SUM(W9:AA9)</f>
+        <v/>
+      </c>
+      <c r="AC9" s="6">
+        <f>D9+J9+P9+V9+AB9</f>
         <v/>
       </c>
     </row>
@@ -1020,53 +1016,65 @@
           <t>Uwaoma Precious</t>
         </is>
       </c>
-      <c r="C10" s="11" t="n"/>
-      <c r="D10" s="11" t="n"/>
-      <c r="E10" s="11" t="n"/>
+      <c r="C10" s="11" t="n">
+        <v>27</v>
+      </c>
+      <c r="D10" s="13">
+        <f>SUM(C10:C10)</f>
+        <v/>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>16.5</v>
+      </c>
       <c r="F10" s="11" t="n"/>
       <c r="G10" s="11" t="n"/>
-      <c r="H10" s="13">
-        <f>SUM(C10:G10)</f>
-        <v/>
-      </c>
+      <c r="H10" s="11" t="n"/>
       <c r="I10" s="11" t="n"/>
-      <c r="J10" s="11" t="n"/>
-      <c r="K10" s="11" t="n"/>
+      <c r="J10" s="13">
+        <f>SUM(E10:I10)</f>
+        <v/>
+      </c>
+      <c r="K10" s="11" t="n">
+        <v>25</v>
+      </c>
       <c r="L10" s="11" t="n"/>
       <c r="M10" s="11" t="n"/>
-      <c r="N10" s="13">
-        <f>SUM(I10:M10)</f>
-        <v/>
-      </c>
+      <c r="N10" s="11" t="n"/>
       <c r="O10" s="11" t="n"/>
-      <c r="P10" s="11" t="n"/>
-      <c r="Q10" s="11" t="n"/>
-      <c r="R10" s="11" t="n"/>
-      <c r="S10" s="11" t="n"/>
-      <c r="T10" s="13">
-        <f>SUM(O10:S10)</f>
-        <v/>
-      </c>
-      <c r="U10" s="11" t="n"/>
-      <c r="V10" s="11" t="n"/>
+      <c r="P10" s="13">
+        <f>SUM(K10:O10)</f>
+        <v/>
+      </c>
+      <c r="Q10" s="11" t="n">
+        <v>41</v>
+      </c>
+      <c r="R10" s="11" t="n">
+        <v>44</v>
+      </c>
+      <c r="S10" s="11" t="n">
+        <v>37</v>
+      </c>
+      <c r="T10" s="11" t="n">
+        <v>17</v>
+      </c>
+      <c r="U10" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="V10" s="13">
+        <f>SUM(Q10:U10)</f>
+        <v/>
+      </c>
       <c r="W10" s="11" t="n"/>
       <c r="X10" s="11" t="n"/>
       <c r="Y10" s="11" t="n"/>
-      <c r="Z10" s="13">
-        <f>SUM(U10:Y10)</f>
-        <v/>
-      </c>
+      <c r="Z10" s="11" t="n"/>
       <c r="AA10" s="11" t="n"/>
-      <c r="AB10" s="11" t="n"/>
-      <c r="AC10" s="11" t="n"/>
-      <c r="AD10" s="11" t="n"/>
-      <c r="AE10" s="11" t="n"/>
-      <c r="AF10" s="13">
-        <f>SUM(AA10:AE10)</f>
-        <v/>
-      </c>
-      <c r="AG10" s="6">
-        <f>H10+N10+T10+Z10+AF10</f>
+      <c r="AB10" s="13">
+        <f>SUM(W10:AA10)</f>
+        <v/>
+      </c>
+      <c r="AC10" s="6">
+        <f>D10+J10+P10+V10+AB10</f>
         <v/>
       </c>
     </row>
@@ -1080,52 +1088,48 @@
         </is>
       </c>
       <c r="C11" s="11" t="n"/>
-      <c r="D11" s="11" t="n"/>
+      <c r="D11" s="13">
+        <f>SUM(C11:C11)</f>
+        <v/>
+      </c>
       <c r="E11" s="11" t="n"/>
       <c r="F11" s="11" t="n"/>
       <c r="G11" s="11" t="n"/>
-      <c r="H11" s="13">
-        <f>SUM(C11:G11)</f>
-        <v/>
-      </c>
+      <c r="H11" s="11" t="n"/>
       <c r="I11" s="11" t="n"/>
-      <c r="J11" s="11" t="n"/>
+      <c r="J11" s="13">
+        <f>SUM(E11:I11)</f>
+        <v/>
+      </c>
       <c r="K11" s="11" t="n"/>
       <c r="L11" s="11" t="n"/>
       <c r="M11" s="11" t="n"/>
-      <c r="N11" s="13">
-        <f>SUM(I11:M11)</f>
-        <v/>
-      </c>
+      <c r="N11" s="11" t="n"/>
       <c r="O11" s="11" t="n"/>
-      <c r="P11" s="11" t="n"/>
+      <c r="P11" s="13">
+        <f>SUM(K11:O11)</f>
+        <v/>
+      </c>
       <c r="Q11" s="11" t="n"/>
       <c r="R11" s="11" t="n"/>
       <c r="S11" s="11" t="n"/>
-      <c r="T11" s="13">
-        <f>SUM(O11:S11)</f>
-        <v/>
-      </c>
+      <c r="T11" s="11" t="n"/>
       <c r="U11" s="11" t="n"/>
-      <c r="V11" s="11" t="n"/>
+      <c r="V11" s="13">
+        <f>SUM(Q11:U11)</f>
+        <v/>
+      </c>
       <c r="W11" s="11" t="n"/>
       <c r="X11" s="11" t="n"/>
       <c r="Y11" s="11" t="n"/>
-      <c r="Z11" s="13">
-        <f>SUM(U11:Y11)</f>
-        <v/>
-      </c>
+      <c r="Z11" s="11" t="n"/>
       <c r="AA11" s="11" t="n"/>
-      <c r="AB11" s="11" t="n"/>
-      <c r="AC11" s="11" t="n"/>
-      <c r="AD11" s="11" t="n"/>
-      <c r="AE11" s="11" t="n"/>
-      <c r="AF11" s="13">
-        <f>SUM(AA11:AE11)</f>
-        <v/>
-      </c>
-      <c r="AG11" s="6">
-        <f>H11+N11+T11+Z11+AF11</f>
+      <c r="AB11" s="13">
+        <f>SUM(W11:AA11)</f>
+        <v/>
+      </c>
+      <c r="AC11" s="6">
+        <f>D11+J11+P11+V11+AB11</f>
         <v/>
       </c>
     </row>
@@ -1139,67 +1143,63 @@
         </is>
       </c>
       <c r="C12" s="11" t="n"/>
-      <c r="D12" s="11" t="n"/>
+      <c r="D12" s="13">
+        <f>SUM(C12:C12)</f>
+        <v/>
+      </c>
       <c r="E12" s="11" t="n"/>
       <c r="F12" s="11" t="n"/>
       <c r="G12" s="11" t="n"/>
-      <c r="H12" s="13">
-        <f>SUM(C12:G12)</f>
-        <v/>
-      </c>
+      <c r="H12" s="11" t="n"/>
       <c r="I12" s="11" t="n"/>
-      <c r="J12" s="11" t="n"/>
+      <c r="J12" s="13">
+        <f>SUM(E12:I12)</f>
+        <v/>
+      </c>
       <c r="K12" s="11" t="n"/>
       <c r="L12" s="11" t="n"/>
       <c r="M12" s="11" t="n"/>
-      <c r="N12" s="13">
-        <f>SUM(I12:M12)</f>
-        <v/>
-      </c>
+      <c r="N12" s="11" t="n"/>
       <c r="O12" s="11" t="n"/>
-      <c r="P12" s="11" t="n"/>
+      <c r="P12" s="13">
+        <f>SUM(K12:O12)</f>
+        <v/>
+      </c>
       <c r="Q12" s="11" t="n"/>
       <c r="R12" s="11" t="n"/>
       <c r="S12" s="11" t="n"/>
-      <c r="T12" s="13">
-        <f>SUM(O12:S12)</f>
-        <v/>
-      </c>
+      <c r="T12" s="11" t="n"/>
       <c r="U12" s="11" t="n"/>
-      <c r="V12" s="11" t="n"/>
+      <c r="V12" s="13">
+        <f>SUM(Q12:U12)</f>
+        <v/>
+      </c>
       <c r="W12" s="11" t="n"/>
       <c r="X12" s="11" t="n"/>
       <c r="Y12" s="11" t="n"/>
-      <c r="Z12" s="13">
-        <f>SUM(U12:Y12)</f>
-        <v/>
-      </c>
+      <c r="Z12" s="11" t="n"/>
       <c r="AA12" s="11" t="n"/>
-      <c r="AB12" s="11" t="n"/>
-      <c r="AC12" s="11" t="n"/>
-      <c r="AD12" s="11" t="n"/>
-      <c r="AE12" s="11" t="n"/>
-      <c r="AF12" s="13">
-        <f>SUM(AA12:AE12)</f>
-        <v/>
-      </c>
-      <c r="AG12" s="6">
-        <f>H12+N12+T12+Z12+AF12</f>
+      <c r="AB12" s="13">
+        <f>SUM(W12:AA12)</f>
+        <v/>
+      </c>
+      <c r="AC12" s="6">
+        <f>D12+J12+P12+V12+AB12</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
-    <mergeCell ref="A1:AG1"/>
+    <mergeCell ref="A1:AC1"/>
     <mergeCell ref="B4:B5"/>
     <mergeCell ref="A4:A5"/>
-    <mergeCell ref="A2:AG2"/>
-    <mergeCell ref="O4:T4"/>
-    <mergeCell ref="AG4:AG5"/>
-    <mergeCell ref="C4:H4"/>
-    <mergeCell ref="U4:Z4"/>
-    <mergeCell ref="AA4:AF4"/>
-    <mergeCell ref="I4:N4"/>
+    <mergeCell ref="K4:P4"/>
+    <mergeCell ref="AC4:AC5"/>
+    <mergeCell ref="Q4:V4"/>
+    <mergeCell ref="W4:AB4"/>
+    <mergeCell ref="E4:J4"/>
+    <mergeCell ref="A2:AC2"/>
+    <mergeCell ref="C4:D4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>